<commit_message>
Fix Excel M3 Quote path for profit≥1
Guard Summary D35/D39 so Quote Total does not #DIV/0! when
profit ≥ 1 (H-bucket guards alone were incomplete).
</commit_message>
<xml_diff>
--- a/excel/BrunoAC_Estimating_UPDATED.xlsx
+++ b/excel/BrunoAC_Estimating_UPDATED.xlsx
@@ -2038,7 +2038,6 @@
         </is>
       </c>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
@@ -2074,7 +2073,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
@@ -9203,6 +9201,7 @@
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="C31" t="inlineStr">
         <is>
@@ -9218,6 +9217,7 @@
         <v/>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="C33" t="inlineStr">
         <is>
@@ -9229,6 +9229,7 @@
         <v/>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="C35" t="inlineStr">
         <is>
@@ -9236,7 +9237,7 @@
         </is>
       </c>
       <c r="D35" s="6">
-        <f>(D33/E11)-D33</f>
+        <f>IF(OR($E$7&gt;=1,$E$11&lt;=0),0,(D33/$E$11)-D33)</f>
         <v/>
       </c>
       <c r="G35">
@@ -9244,6 +9245,9 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39">
       <c r="C39" s="21" t="inlineStr">
         <is>
@@ -9251,7 +9255,7 @@
         </is>
       </c>
       <c r="D39" s="9">
-        <f>D33+D35</f>
+        <f>IF(OR($E$7&gt;=1,$E$11&lt;=0),D28,D33+D35)</f>
         <v/>
       </c>
       <c r="E39" t="inlineStr">

</xml_diff>